<commit_message>
alterações, criação dos gráficos das tef, imputacao pela idade da mae
</commit_message>
<xml_diff>
--- a/202505_resultados/2022_TEF_TFT_Fluxos.xlsx
+++ b/202505_resultados/2022_TEF_TFT_Fluxos.xlsx
@@ -419,37 +419,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0,0056</t>
+          <t>0,0054</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,0602</t>
+          <t>0,0611</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,0800</t>
+          <t>0,0799</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,0826</t>
+          <t>0,0813</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0,0577</t>
+          <t>0,0582</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0,0216</t>
+          <t>0,0219</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0,0052</t>
+          <t>0,0050</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -471,42 +471,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>0,0037</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0,0900</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0,1026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0,0969</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0,0608</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0,0176</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>0,0043</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0,0896</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0,1038</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0,0959</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0,0580</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0,0193</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0,0052</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0,0020</t>
+          <t>0,0019</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -523,42 +523,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0,0064</t>
+          <t>0,0059</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,0663</t>
+          <t>0,0686</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,0807</t>
+          <t>0,0828</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,0869</t>
+          <t>0,0816</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0,0588</t>
+          <t>0,0598</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0,0179</t>
+          <t>0,0183</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0,0030</t>
+          <t>0,0027</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0,0011</t>
+          <t>0,0010</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -575,37 +575,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0,0051</t>
+          <t>0,0053</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,0508</t>
+          <t>0,0507</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,0732</t>
+          <t>0,0727</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,0769</t>
+          <t>0,0770</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0,0566</t>
+          <t>0,0562</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0,0233</t>
+          <t>0,0242</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0,0057</t>
+          <t>0,0056</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -627,17 +627,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0,0060</t>
+          <t>0,0061</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,0527</t>
+          <t>0,0530</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,0751</t>
+          <t>0,0745</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,0577</t>
+          <t>0,0582</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0,0251</t>
+          <t>0,0250</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0,0075</t>
+          <t>0,0073</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0,0011</t>
+          <t>0,0010</t>
         </is>
       </c>
     </row>
@@ -679,37 +679,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0,0061</t>
+          <t>0,0058</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0,0616</t>
+          <t>0,0647</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,0917</t>
+          <t>0,0895</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0,0865</t>
+          <t>0,0855</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,0597</t>
+          <t>0,0606</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0,0206</t>
+          <t>0,0202</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0,0053</t>
+          <t>0,0052</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0,0012</t>
+          <t>0,0010</t>
         </is>
       </c>
     </row>
@@ -736,32 +736,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0,0669</t>
+          <t>0,0662</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,0956</t>
+          <t>0,0966</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0,1096</t>
+          <t>0,1087</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,0533</t>
+          <t>0,0541</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0,0197</t>
+          <t>0,0192</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0,0045</t>
+          <t>0,0047</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -783,32 +783,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0,0041</t>
+          <t>0,0058</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0,0859</t>
+          <t>0,1041</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,1143</t>
+          <t>0,0990</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0,0954</t>
+          <t>0,0836</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0,0723</t>
+          <t>0,0789</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0,0229</t>
+          <t>0,0195</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0,0009</t>
+          <t>0,0008</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -835,42 +835,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0,0066</t>
+          <t>0,0058</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0,1037</t>
+          <t>0,1131</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,1124</t>
+          <t>0,1031</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0,0938</t>
+          <t>0,0965</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0,0663</t>
+          <t>0,0618</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0,0212</t>
+          <t>0,0245</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0,0068</t>
+          <t>0,0051</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0,0024</t>
+          <t>0,0023</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -887,42 +887,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0,0076</t>
+          <t>0,0042</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0,0840</t>
+          <t>0,1020</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,1377</t>
+          <t>0,1408</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,1177</t>
+          <t>0,1091</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0,0538</t>
+          <t>0,0603</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0,0490</t>
+          <t>0,0301</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0,0098</t>
+          <t>0,0067</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0,0020</t>
+          <t>0,0015</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -944,37 +944,37 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0,0907</t>
+          <t>0,0856</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,0988</t>
+          <t>0,0992</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0,0897</t>
+          <t>0,0911</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0,0517</t>
+          <t>0,0588</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0,0170</t>
+          <t>0,0142</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0,0041</t>
+          <t>0,0036</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0,0019</t>
+          <t>0,0018</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -991,42 +991,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0,0052</t>
+          <t>0,0013</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0,0791</t>
+          <t>0,0654</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,1144</t>
+          <t>0,1401</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0,1196</t>
+          <t>0,1165</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0,0687</t>
+          <t>0,0743</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0,0088</t>
+          <t>0,0026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0,0123</t>
+          <t>0,0072</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0,0015</t>
+          <t>0,0006</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1043,32 +1043,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0,0063</t>
+          <t>0,0034</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0,0768</t>
+          <t>0,0734</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,0893</t>
+          <t>0,0903</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0,0981</t>
+          <t>0,1089</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0,0655</t>
+          <t>0,0615</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0,0180</t>
+          <t>0,0174</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0,0026</t>
+          <t>0,0018</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1095,37 +1095,37 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>0,0017</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0,0824</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0,0982</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0,1006</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0,0518</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0,0118</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>0,0025</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0,0918</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>0,0892</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>0,0987</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0,0526</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>0,0105</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0,0026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1147,42 +1147,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0,0056</t>
+          <t>0,0088</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0,0624</t>
+          <t>0,0666</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,0871</t>
+          <t>0,0707</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0,0877</t>
+          <t>0,0907</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0,0654</t>
+          <t>0,0683</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0,0131</t>
+          <t>0,0165</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0,0034</t>
+          <t>0,0024</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>0,0006</t>
+          <t>0,0005</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1199,37 +1199,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>0,0015</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0,0633</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0,0751</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0,0836</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0,0584</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0,0212</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>0,0020</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>0,0609</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0,0770</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0,0874</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0,0577</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>0,0172</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0,0024</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1251,37 +1251,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0,0031</t>
+          <t>0,0037</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0,0502</t>
+          <t>0,0467</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,0759</t>
+          <t>0,0867</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0,0824</t>
+          <t>0,0696</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0,0587</t>
+          <t>0,0640</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0,0203</t>
+          <t>0,0195</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0,0036</t>
+          <t>0,0041</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0,0007</t>
+          <t>0,0005</t>
         </is>
       </c>
     </row>
@@ -1303,37 +1303,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0,0034</t>
+          <t>0,0012</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0,0635</t>
+          <t>0,0731</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,0864</t>
+          <t>0,0833</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0,0932</t>
+          <t>0,0875</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0,0586</t>
+          <t>0,0570</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0,0173</t>
+          <t>0,0205</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0,0033</t>
+          <t>0,0027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1355,37 +1355,37 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0,0203</t>
+          <t>0,0212</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0,0757</t>
+          <t>0,0689</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,0735</t>
+          <t>0,0847</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0,0764</t>
+          <t>0,0717</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0,0559</t>
+          <t>0,0583</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0,0168</t>
+          <t>0,0141</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0,0021</t>
+          <t>0,0023</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1407,37 +1407,37 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0,0029</t>
+          <t>0,0013</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0,0866</t>
+          <t>0,0937</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,0980</t>
+          <t>0,1006</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0,0973</t>
+          <t>0,0958</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0,0647</t>
+          <t>0,0572</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0,0186</t>
+          <t>0,0190</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0,0022</t>
+          <t>0,0016</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1459,42 +1459,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0,0102</t>
+          <t>0,0023</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0,0421</t>
+          <t>0,0527</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,0893</t>
+          <t>0,0842</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0,0880</t>
+          <t>0,0890</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0,0671</t>
+          <t>0,0728</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0,0206</t>
+          <t>0,0179</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0,0038</t>
+          <t>0,0021</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>0,0017</t>
+          <t>0,0011</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1511,32 +1511,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0,0041</t>
+          <t>0,0036</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0,0548</t>
+          <t>0,0655</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,0764</t>
+          <t>0,0766</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0,0842</t>
+          <t>0,0723</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0,0601</t>
+          <t>0,0616</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0,0220</t>
+          <t>0,0212</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1563,37 +1563,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0,0043</t>
+          <t>0,0042</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0,0508</t>
+          <t>0,0512</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,0701</t>
+          <t>0,0692</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0,0776</t>
+          <t>0,0779</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0,0562</t>
+          <t>0,0561</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0,0234</t>
+          <t>0,0238</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0,0055</t>
+          <t>0,0053</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1615,32 +1615,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0,0040</t>
+          <t>0,0033</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0,0584</t>
+          <t>0,0538</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,0831</t>
+          <t>0,0938</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0,0862</t>
+          <t>0,0806</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0,0714</t>
+          <t>0,0736</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0,0241</t>
+          <t>0,0223</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0,0021</t>
+          <t>0,0020</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1667,42 +1667,42 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0,0076</t>
+          <t>0,0068</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0,0537</t>
+          <t>0,0544</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,0747</t>
+          <t>0,0719</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0,0706</t>
+          <t>0,0726</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0,0484</t>
+          <t>0,0494</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0,0223</t>
+          <t>0,0224</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0,0060</t>
+          <t>0,0058</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0,0024</t>
+          <t>0,0025</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0,0048</t>
+          <t>0,0054</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0,0490</t>
+          <t>0,0487</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0,0733</t>
+          <t>0,0728</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1739,17 +1739,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0,0584</t>
+          <t>0,0570</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0,0236</t>
+          <t>0,0251</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0,0057</t>
+          <t>0,0056</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1776,22 +1776,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0,0561</t>
+          <t>0,0562</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0,0787</t>
+          <t>0,0783</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0,0818</t>
+          <t>0,0820</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0,0571</t>
+          <t>0,0570</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1828,32 +1828,32 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>0,0532</t>
+          <t>0,0543</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0,0769</t>
+          <t>0,0751</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0,0835</t>
+          <t>0,0844</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0,0626</t>
+          <t>0,0631</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0,0198</t>
+          <t>0,0200</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0,0056</t>
+          <t>0,0047</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>0,0007</t>
+          <t>0,0005</t>
         </is>
       </c>
     </row>
@@ -1875,12 +1875,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0,0058</t>
+          <t>0,0060</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0,0487</t>
+          <t>0,0486</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1890,17 +1890,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0,0763</t>
+          <t>0,0754</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0,0544</t>
+          <t>0,0556</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0,0283</t>
+          <t>0,0279</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0,0125</t>
+          <t>0,0117</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0,0763</t>
+          <t>0,0771</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1942,22 +1942,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0,0872</t>
+          <t>0,0873</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0,0605</t>
+          <t>0,0612</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0,0254</t>
+          <t>0,0247</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0,0094</t>
+          <t>0,0093</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1979,42 +1979,42 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0,0042</t>
+          <t>0,0022</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0,0797</t>
+          <t>0,0903</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0,1072</t>
+          <t>0,0992</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0,1039</t>
+          <t>0,1013</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0,0632</t>
+          <t>0,0653</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0,0148</t>
+          <t>0,0150</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0,0030</t>
+          <t>0,0031</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0,0014</t>
+          <t>0,0013</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2031,42 +2031,42 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0,0031</t>
+          <t>0,0032</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0,0538</t>
+          <t>0,0528</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0,0919</t>
+          <t>0,0929</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0,0806</t>
+          <t>0,0814</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0,0559</t>
+          <t>0,0556</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0,0174</t>
+          <t>0,0169</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0,0043</t>
+          <t>0,0042</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0,0018</t>
+          <t>0,0017</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2083,32 +2083,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0,0093</t>
+          <t>0,0106</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0,0435</t>
+          <t>0,0492</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0,0720</t>
+          <t>0,0681</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0,0772</t>
+          <t>0,0729</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0,0638</t>
+          <t>0,0665</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>0,0313</t>
+          <t>0,0305</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>0,0022</t>
+          <t>0,0011</t>
         </is>
       </c>
     </row>
@@ -2196,25 +2196,25 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.0045</v>
+        <v>0.0042</v>
       </c>
       <c r="C2">
-        <v>0.0606</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="D2">
-        <v>0.0818</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="E2">
-        <v>0.0823</v>
+        <v>0.0824</v>
       </c>
       <c r="F2">
-        <v>0.0565</v>
+        <v>0.0568</v>
       </c>
       <c r="G2">
-        <v>0.0221</v>
+        <v>0.0226</v>
       </c>
       <c r="H2">
-        <v>0.0051</v>
+        <v>0.005</v>
       </c>
       <c r="I2">
         <v>0.0019</v>
@@ -2230,28 +2230,28 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.0038</v>
+        <v>0.0035</v>
       </c>
       <c r="C3">
-        <v>0.0863</v>
+        <v>0.0866</v>
       </c>
       <c r="D3">
-        <v>0.107</v>
+        <v>0.1012</v>
       </c>
       <c r="E3">
-        <v>0.0979</v>
+        <v>0.0973</v>
       </c>
       <c r="F3">
-        <v>0.0587</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="G3">
-        <v>0.0184</v>
+        <v>0.0202</v>
       </c>
       <c r="H3">
-        <v>0.0043</v>
+        <v>0.004</v>
       </c>
       <c r="I3">
-        <v>0.0019</v>
+        <v>0.0018</v>
       </c>
       <c r="J3">
         <v>0.001</v>
@@ -2264,25 +2264,25 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.0033</v>
+        <v>0.0032</v>
       </c>
       <c r="C4">
-        <v>0.0687</v>
+        <v>0.0726</v>
       </c>
       <c r="D4">
-        <v>0.0867</v>
+        <v>0.0827</v>
       </c>
       <c r="E4">
         <v>0.0844</v>
       </c>
       <c r="F4">
-        <v>0.0561</v>
+        <v>0.0546</v>
       </c>
       <c r="G4">
-        <v>0.0181</v>
+        <v>0.0199</v>
       </c>
       <c r="H4">
-        <v>0.0028</v>
+        <v>0.0025</v>
       </c>
       <c r="I4">
         <v>0.001</v>
@@ -2298,22 +2298,22 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.0051</v>
+        <v>0.0044</v>
       </c>
       <c r="C5">
-        <v>0.0512</v>
+        <v>0.052</v>
       </c>
       <c r="D5">
-        <v>0.073</v>
+        <v>0.0722</v>
       </c>
       <c r="E5">
-        <v>0.07729999999999999</v>
+        <v>0.0774</v>
       </c>
       <c r="F5">
-        <v>0.0553</v>
+        <v>0.0556</v>
       </c>
       <c r="G5">
-        <v>0.0242</v>
+        <v>0.0243</v>
       </c>
       <c r="H5">
         <v>0.0057</v>
@@ -2341,13 +2341,13 @@
         <v>0.0745</v>
       </c>
       <c r="E6">
-        <v>0.0806</v>
+        <v>0.0804</v>
       </c>
       <c r="F6">
-        <v>0.0568</v>
+        <v>0.0572</v>
       </c>
       <c r="G6">
-        <v>0.0263</v>
+        <v>0.026</v>
       </c>
       <c r="H6">
         <v>0.0074</v>
@@ -2366,25 +2366,25 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.0044</v>
+        <v>0.0052</v>
       </c>
       <c r="C7">
-        <v>0.0606</v>
+        <v>0.06809999999999999</v>
       </c>
       <c r="D7">
-        <v>0.09320000000000001</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="E7">
-        <v>0.0856</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="F7">
-        <v>0.061</v>
+        <v>0.0613</v>
       </c>
       <c r="G7">
-        <v>0.0213</v>
+        <v>0.0194</v>
       </c>
       <c r="H7">
-        <v>0.0056</v>
+        <v>0.0054</v>
       </c>
       <c r="I7">
         <v>0.0021</v>
@@ -2463,12 +2463,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0,0047</t>
+          <t>0,0048</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,0640</t>
+          <t>0,0639</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2483,12 +2483,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0,0557</t>
+          <t>0,0556</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0,0228</t>
+          <t>0,0230</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1,90</t>
+          <t>1,89</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2,01</t>
+          <t>1,99</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2,31</t>
+          <t>2,28</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2,05</t>
+          <t>2,04</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1,63</t>
+          <t>1,62</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1,64</t>
+          <t>1,63</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1,86</t>
+          <t>1,85</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1,62</t>
+          <t>1,61</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1,54</t>
+          <t>1,53</t>
         </is>
       </c>
     </row>

</xml_diff>